<commit_message>
Update lotto data (2026-03-07 13:14)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47622,25 +47622,25 @@
       <c r="A1214" s="31" t="n">
         <v>1213</v>
       </c>
-      <c r="B1214" t="n">
+      <c r="B1214" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="C1214" t="n">
+      <c r="C1214" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="D1214" t="n">
+      <c r="D1214" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="E1214" t="n">
+      <c r="E1214" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="F1214" t="n">
+      <c r="F1214" s="27" t="n">
         <v>36</v>
       </c>
-      <c r="G1214" t="n">
+      <c r="G1214" s="27" t="n">
         <v>38</v>
       </c>
-      <c r="H1214" t="n">
+      <c r="H1214" s="27" t="n">
         <v>2</v>
       </c>
       <c r="J1214" s="27">
@@ -47657,7 +47657,30 @@
       </c>
     </row>
     <row r="1215" ht="13.8" customHeight="1" s="28">
-      <c r="A1215" s="31" t="n"/>
+      <c r="A1215" s="31" t="n">
+        <v>1214</v>
+      </c>
+      <c r="B1215" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1215" t="n">
+        <v>11</v>
+      </c>
+      <c r="D1215" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>27</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>36</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1215" t="n">
+        <v>2</v>
+      </c>
       <c r="J1215" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1215:G1215, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-03-21 13:24)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -905,7 +905,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1108,7 +1108,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1163,7 +1163,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -47698,25 +47698,25 @@
       <c r="A1216" s="31" t="n">
         <v>1215</v>
       </c>
-      <c r="B1216" t="n">
+      <c r="B1216" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="C1216" t="n">
+      <c r="C1216" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="D1216" t="n">
+      <c r="D1216" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="E1216" t="n">
+      <c r="E1216" s="27" t="n">
         <v>21</v>
       </c>
-      <c r="F1216" t="n">
+      <c r="F1216" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="G1216" t="n">
+      <c r="G1216" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="H1216" t="n">
+      <c r="H1216" s="27" t="n">
         <v>39</v>
       </c>
       <c r="J1216" s="27">
@@ -47733,7 +47733,30 @@
       </c>
     </row>
     <row r="1217" ht="13.8" customHeight="1" s="28">
-      <c r="A1217" s="31" t="n"/>
+      <c r="A1217" s="31" t="n">
+        <v>1216</v>
+      </c>
+      <c r="B1217" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1217" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1217" t="n">
+        <v>14</v>
+      </c>
+      <c r="E1217" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1217" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1217" t="n">
+        <v>24</v>
+      </c>
+      <c r="H1217" t="n">
+        <v>25</v>
+      </c>
       <c r="J1217" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1217:G1217, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-03-28 13:31)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47736,25 +47736,25 @@
       <c r="A1217" s="31" t="n">
         <v>1216</v>
       </c>
-      <c r="B1217" t="n">
+      <c r="B1217" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="C1217" t="n">
+      <c r="C1217" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="D1217" t="n">
+      <c r="D1217" s="27" t="n">
         <v>14</v>
       </c>
-      <c r="E1217" t="n">
+      <c r="E1217" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="F1217" t="n">
+      <c r="F1217" s="27" t="n">
         <v>23</v>
       </c>
-      <c r="G1217" t="n">
+      <c r="G1217" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="H1217" t="n">
+      <c r="H1217" s="27" t="n">
         <v>25</v>
       </c>
       <c r="J1217" s="27">
@@ -47771,7 +47771,30 @@
       </c>
     </row>
     <row r="1218" ht="13.8" customHeight="1" s="28">
-      <c r="A1218" s="31" t="n"/>
+      <c r="A1218" s="31" t="n">
+        <v>1217</v>
+      </c>
+      <c r="B1218" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1218" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1218" t="n">
+        <v>15</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>20</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>31</v>
+      </c>
+      <c r="H1218" t="n">
+        <v>41</v>
+      </c>
       <c r="J1218" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1218:G1218, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-04-04 13:33)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47774,25 +47774,25 @@
       <c r="A1218" s="31" t="n">
         <v>1217</v>
       </c>
-      <c r="B1218" t="n">
+      <c r="B1218" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="C1218" t="n">
+      <c r="C1218" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="D1218" t="n">
+      <c r="D1218" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="E1218" t="n">
+      <c r="E1218" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="F1218" t="n">
+      <c r="F1218" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="G1218" t="n">
+      <c r="G1218" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="H1218" t="n">
+      <c r="H1218" s="27" t="n">
         <v>41</v>
       </c>
       <c r="J1218" s="27">
@@ -47809,7 +47809,30 @@
       </c>
     </row>
     <row r="1219" ht="13.8" customHeight="1" s="28">
-      <c r="A1219" s="31" t="n"/>
+      <c r="A1219" s="31" t="n">
+        <v>1218</v>
+      </c>
+      <c r="B1219" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1219" t="n">
+        <v>28</v>
+      </c>
+      <c r="D1219" t="n">
+        <v>31</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>32</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>42</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>45</v>
+      </c>
+      <c r="H1219" t="n">
+        <v>25</v>
+      </c>
       <c r="J1219" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1219:G1219, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-04-11 13:35)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47812,25 +47812,25 @@
       <c r="A1219" s="31" t="n">
         <v>1218</v>
       </c>
-      <c r="B1219" t="n">
+      <c r="B1219" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="C1219" t="n">
+      <c r="C1219" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="D1219" t="n">
+      <c r="D1219" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="E1219" t="n">
+      <c r="E1219" s="27" t="n">
         <v>32</v>
       </c>
-      <c r="F1219" t="n">
+      <c r="F1219" s="27" t="n">
         <v>42</v>
       </c>
-      <c r="G1219" t="n">
+      <c r="G1219" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="H1219" t="n">
+      <c r="H1219" s="27" t="n">
         <v>25</v>
       </c>
       <c r="J1219" s="27">
@@ -47847,7 +47847,30 @@
       </c>
     </row>
     <row r="1220" ht="13.8" customHeight="1" s="28">
-      <c r="A1220" s="31" t="n"/>
+      <c r="A1220" s="31" t="n">
+        <v>1219</v>
+      </c>
+      <c r="B1220" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1220" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1220" t="n">
+        <v>15</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>28</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>39</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>45</v>
+      </c>
+      <c r="H1220" t="n">
+        <v>31</v>
+      </c>
       <c r="J1220" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1220:G1220, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-04-18 13:39)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47850,25 +47850,25 @@
       <c r="A1220" s="31" t="n">
         <v>1219</v>
       </c>
-      <c r="B1220" t="n">
+      <c r="B1220" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="C1220" t="n">
+      <c r="C1220" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="D1220" t="n">
+      <c r="D1220" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="E1220" t="n">
+      <c r="E1220" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="F1220" t="n">
+      <c r="F1220" s="27" t="n">
         <v>39</v>
       </c>
-      <c r="G1220" t="n">
+      <c r="G1220" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="H1220" t="n">
+      <c r="H1220" s="27" t="n">
         <v>31</v>
       </c>
       <c r="J1220" s="27">
@@ -47885,7 +47885,30 @@
       </c>
     </row>
     <row r="1221" ht="13.8" customHeight="1" s="28">
-      <c r="A1221" s="31" t="n"/>
+      <c r="A1221" s="31" t="n">
+        <v>1220</v>
+      </c>
+      <c r="B1221" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1221" t="n">
+        <v>22</v>
+      </c>
+      <c r="D1221" t="n">
+        <v>25</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>28</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>34</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>43</v>
+      </c>
+      <c r="H1221" t="n">
+        <v>16</v>
+      </c>
       <c r="J1221" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1221:G1221, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-04-25 13:42)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47888,25 +47888,25 @@
       <c r="A1221" s="31" t="n">
         <v>1220</v>
       </c>
-      <c r="B1221" t="n">
+      <c r="B1221" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="C1221" t="n">
+      <c r="C1221" s="27" t="n">
         <v>22</v>
       </c>
-      <c r="D1221" t="n">
+      <c r="D1221" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="E1221" t="n">
+      <c r="E1221" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="F1221" t="n">
+      <c r="F1221" s="27" t="n">
         <v>34</v>
       </c>
-      <c r="G1221" t="n">
+      <c r="G1221" s="27" t="n">
         <v>43</v>
       </c>
-      <c r="H1221" t="n">
+      <c r="H1221" s="27" t="n">
         <v>16</v>
       </c>
       <c r="J1221" s="27">
@@ -47923,7 +47923,30 @@
       </c>
     </row>
     <row r="1222" ht="13.8" customHeight="1" s="28">
-      <c r="A1222" s="31" t="n"/>
+      <c r="A1222" s="31" t="n">
+        <v>1221</v>
+      </c>
+      <c r="B1222" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1222" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1222" t="n">
+        <v>18</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>28</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1222" t="n">
+        <v>9</v>
+      </c>
       <c r="J1222" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1222:G1222, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-05-02 13:52)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47926,25 +47926,25 @@
       <c r="A1222" s="31" t="n">
         <v>1221</v>
       </c>
-      <c r="B1222" t="n">
+      <c r="B1222" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="C1222" t="n">
+      <c r="C1222" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1222" t="n">
+      <c r="D1222" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="E1222" t="n">
+      <c r="E1222" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="F1222" t="n">
+      <c r="F1222" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="G1222" t="n">
+      <c r="G1222" s="27" t="n">
         <v>36</v>
       </c>
-      <c r="H1222" t="n">
+      <c r="H1222" s="27" t="n">
         <v>9</v>
       </c>
       <c r="J1222" s="27">
@@ -47961,7 +47961,30 @@
       </c>
     </row>
     <row r="1223" ht="13.8" customHeight="1" s="28">
-      <c r="A1223" s="31" t="n"/>
+      <c r="A1223" s="31" t="n">
+        <v>1222</v>
+      </c>
+      <c r="B1223" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1223" t="n">
+        <v>11</v>
+      </c>
+      <c r="D1223" t="n">
+        <v>17</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>22</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>41</v>
+      </c>
+      <c r="H1223" t="n">
+        <v>34</v>
+      </c>
       <c r="J1223" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1223:G1223, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-05-09 13:57)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -47964,25 +47964,25 @@
       <c r="A1223" s="31" t="n">
         <v>1222</v>
       </c>
-      <c r="B1223" t="n">
+      <c r="B1223" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="C1223" t="n">
+      <c r="C1223" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="D1223" t="n">
+      <c r="D1223" s="27" t="n">
         <v>17</v>
       </c>
-      <c r="E1223" t="n">
+      <c r="E1223" s="27" t="n">
         <v>22</v>
       </c>
-      <c r="F1223" t="n">
+      <c r="F1223" s="27" t="n">
         <v>32</v>
       </c>
-      <c r="G1223" t="n">
+      <c r="G1223" s="27" t="n">
         <v>41</v>
       </c>
-      <c r="H1223" t="n">
+      <c r="H1223" s="27" t="n">
         <v>34</v>
       </c>
       <c r="J1223" s="27">
@@ -47999,7 +47999,30 @@
       </c>
     </row>
     <row r="1224" ht="13.8" customHeight="1" s="28">
-      <c r="A1224" s="31" t="n"/>
+      <c r="A1224" s="31" t="n">
+        <v>1223</v>
+      </c>
+      <c r="B1224" t="n">
+        <v>16</v>
+      </c>
+      <c r="C1224" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1224" t="n">
+        <v>20</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>32</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>33</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>39</v>
+      </c>
+      <c r="H1224" t="n">
+        <v>26</v>
+      </c>
       <c r="J1224" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1224:G1224, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-05-16 14:04)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48002,25 +48002,25 @@
       <c r="A1224" s="31" t="n">
         <v>1223</v>
       </c>
-      <c r="B1224" t="n">
+      <c r="B1224" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="C1224" t="n">
+      <c r="C1224" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="D1224" t="n">
+      <c r="D1224" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E1224" t="n">
+      <c r="E1224" s="27" t="n">
         <v>32</v>
       </c>
-      <c r="F1224" t="n">
+      <c r="F1224" s="27" t="n">
         <v>33</v>
       </c>
-      <c r="G1224" t="n">
+      <c r="G1224" s="27" t="n">
         <v>39</v>
       </c>
-      <c r="H1224" t="n">
+      <c r="H1224" s="27" t="n">
         <v>26</v>
       </c>
       <c r="J1224" s="27">
@@ -48037,7 +48037,30 @@
       </c>
     </row>
     <row r="1225" ht="13.8" customHeight="1" s="28">
-      <c r="A1225" s="31" t="n"/>
+      <c r="A1225" s="31" t="n">
+        <v>1224</v>
+      </c>
+      <c r="B1225" t="n">
+        <v>9</v>
+      </c>
+      <c r="C1225" t="n">
+        <v>18</v>
+      </c>
+      <c r="D1225" t="n">
+        <v>21</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>27</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>44</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>45</v>
+      </c>
+      <c r="H1225" t="n">
+        <v>28</v>
+      </c>
       <c r="J1225" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1225:G1225, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-05-23 14:08)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48040,25 +48040,25 @@
       <c r="A1225" s="31" t="n">
         <v>1224</v>
       </c>
-      <c r="B1225" t="n">
+      <c r="B1225" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="C1225" t="n">
+      <c r="C1225" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="D1225" t="n">
+      <c r="D1225" s="27" t="n">
         <v>21</v>
       </c>
-      <c r="E1225" t="n">
+      <c r="E1225" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="F1225" t="n">
+      <c r="F1225" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="G1225" t="n">
+      <c r="G1225" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="H1225" t="n">
+      <c r="H1225" s="27" t="n">
         <v>28</v>
       </c>
       <c r="J1225" s="27">
@@ -48075,7 +48075,30 @@
       </c>
     </row>
     <row r="1226" ht="13.8" customHeight="1" s="28">
-      <c r="A1226" s="31" t="n"/>
+      <c r="A1226" s="31" t="n">
+        <v>1225</v>
+      </c>
+      <c r="B1226" t="n">
+        <v>8</v>
+      </c>
+      <c r="C1226" t="n">
+        <v>9</v>
+      </c>
+      <c r="D1226" t="n">
+        <v>19</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>41</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1226" t="n">
+        <v>33</v>
+      </c>
       <c r="J1226" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1226:G1226, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-05-30 14:12)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48078,25 +48078,25 @@
       <c r="A1226" s="31" t="n">
         <v>1225</v>
       </c>
-      <c r="B1226" t="n">
+      <c r="B1226" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="C1226" t="n">
+      <c r="C1226" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="D1226" t="n">
+      <c r="D1226" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="E1226" t="n">
+      <c r="E1226" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="F1226" t="n">
+      <c r="F1226" s="27" t="n">
         <v>41</v>
       </c>
-      <c r="G1226" t="n">
+      <c r="G1226" s="27" t="n">
         <v>42</v>
       </c>
-      <c r="H1226" t="n">
+      <c r="H1226" s="27" t="n">
         <v>33</v>
       </c>
       <c r="J1226" s="27">
@@ -48113,7 +48113,30 @@
       </c>
     </row>
     <row r="1227" ht="13.8" customHeight="1" s="28">
-      <c r="A1227" s="31" t="n"/>
+      <c r="A1227" s="31" t="n">
+        <v>1226</v>
+      </c>
+      <c r="B1227" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1227" t="n">
+        <v>6</v>
+      </c>
+      <c r="D1227" t="n">
+        <v>13</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>17</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>26</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1227" t="n">
+        <v>41</v>
+      </c>
       <c r="J1227" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1227:G1227, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-06-06 14:15)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48116,25 +48116,25 @@
       <c r="A1227" s="31" t="n">
         <v>1226</v>
       </c>
-      <c r="B1227" t="n">
+      <c r="B1227" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="C1227" t="n">
+      <c r="C1227" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="D1227" t="n">
+      <c r="D1227" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="E1227" t="n">
+      <c r="E1227" s="27" t="n">
         <v>17</v>
       </c>
-      <c r="F1227" t="n">
+      <c r="F1227" s="27" t="n">
         <v>26</v>
       </c>
-      <c r="G1227" t="n">
+      <c r="G1227" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="H1227" t="n">
+      <c r="H1227" s="27" t="n">
         <v>41</v>
       </c>
       <c r="J1227" s="27">
@@ -48151,7 +48151,30 @@
       </c>
     </row>
     <row r="1228" ht="13.8" customHeight="1" s="28">
-      <c r="A1228" s="31" t="n"/>
+      <c r="A1228" s="31" t="n">
+        <v>1227</v>
+      </c>
+      <c r="B1228" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1228" t="n">
+        <v>14</v>
+      </c>
+      <c r="D1228" t="n">
+        <v>16</v>
+      </c>
+      <c r="E1228" t="n">
+        <v>34</v>
+      </c>
+      <c r="F1228" t="n">
+        <v>41</v>
+      </c>
+      <c r="G1228" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1228" t="n">
+        <v>13</v>
+      </c>
       <c r="J1228" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1228:G1228, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-06-13 14:37)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48154,25 +48154,25 @@
       <c r="A1228" s="31" t="n">
         <v>1227</v>
       </c>
-      <c r="B1228" t="n">
+      <c r="B1228" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="C1228" t="n">
+      <c r="C1228" s="27" t="n">
         <v>14</v>
       </c>
-      <c r="D1228" t="n">
+      <c r="D1228" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="E1228" t="n">
+      <c r="E1228" s="27" t="n">
         <v>34</v>
       </c>
-      <c r="F1228" t="n">
+      <c r="F1228" s="27" t="n">
         <v>41</v>
       </c>
-      <c r="G1228" t="n">
+      <c r="G1228" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="H1228" t="n">
+      <c r="H1228" s="27" t="n">
         <v>13</v>
       </c>
       <c r="J1228" s="27">
@@ -48189,7 +48189,30 @@
       </c>
     </row>
     <row r="1229" ht="13.8" customHeight="1" s="28">
-      <c r="A1229" s="31" t="n"/>
+      <c r="A1229" s="31" t="n">
+        <v>1228</v>
+      </c>
+      <c r="B1229" t="n">
+        <v>24</v>
+      </c>
+      <c r="C1229" t="n">
+        <v>29</v>
+      </c>
+      <c r="D1229" t="n">
+        <v>30</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>31</v>
+      </c>
+      <c r="F1229" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1229" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1229" t="n">
+        <v>1</v>
+      </c>
       <c r="J1229" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1229:G1229, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-06-20 14:40)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48192,25 +48192,25 @@
       <c r="A1229" s="31" t="n">
         <v>1228</v>
       </c>
-      <c r="B1229" t="n">
+      <c r="B1229" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="C1229" t="n">
+      <c r="C1229" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="D1229" t="n">
+      <c r="D1229" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="E1229" t="n">
+      <c r="E1229" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="F1229" t="n">
+      <c r="F1229" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="G1229" t="n">
+      <c r="G1229" s="27" t="n">
         <v>44</v>
       </c>
-      <c r="H1229" t="n">
+      <c r="H1229" s="27" t="n">
         <v>1</v>
       </c>
       <c r="J1229" s="27">
@@ -48227,7 +48227,30 @@
       </c>
     </row>
     <row r="1230" ht="13.8" customHeight="1" s="28">
-      <c r="A1230" s="31" t="n"/>
+      <c r="A1230" s="31" t="n">
+        <v>1229</v>
+      </c>
+      <c r="B1230" t="n">
+        <v>12</v>
+      </c>
+      <c r="C1230" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1230" t="n">
+        <v>29</v>
+      </c>
+      <c r="E1230" t="n">
+        <v>34</v>
+      </c>
+      <c r="F1230" t="n">
+        <v>37</v>
+      </c>
+      <c r="G1230" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1230" t="n">
+        <v>16</v>
+      </c>
       <c r="J1230" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1230:G1230, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>

<commit_message>
Update lotto data (2026-06-27 14:12)
</commit_message>
<xml_diff>
--- a/lotto_prob.xlsx
+++ b/lotto_prob.xlsx
@@ -48230,25 +48230,25 @@
       <c r="A1230" s="31" t="n">
         <v>1229</v>
       </c>
-      <c r="B1230" t="n">
+      <c r="B1230" s="27" t="n">
         <v>12</v>
       </c>
-      <c r="C1230" t="n">
+      <c r="C1230" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="D1230" t="n">
+      <c r="D1230" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="E1230" t="n">
+      <c r="E1230" s="27" t="n">
         <v>34</v>
       </c>
-      <c r="F1230" t="n">
+      <c r="F1230" s="27" t="n">
         <v>37</v>
       </c>
-      <c r="G1230" t="n">
+      <c r="G1230" s="27" t="n">
         <v>42</v>
       </c>
-      <c r="H1230" t="n">
+      <c r="H1230" s="27" t="n">
         <v>16</v>
       </c>
       <c r="J1230" s="27">
@@ -48265,7 +48265,30 @@
       </c>
     </row>
     <row r="1231" ht="13.8" customHeight="1" s="28">
-      <c r="A1231" s="31" t="n"/>
+      <c r="A1231" s="31" t="n">
+        <v>1230</v>
+      </c>
+      <c r="B1231" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1231" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1231" t="n">
+        <v>9</v>
+      </c>
+      <c r="E1231" t="n">
+        <v>22</v>
+      </c>
+      <c r="F1231" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1231" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1231" t="n">
+        <v>45</v>
+      </c>
       <c r="J1231" s="27">
         <f>SUMPRODUCT(COUNTIFS(확률!$J$2:$J$46, 원본!B1231:G1231, 확률!$M$2:$M$46, "&lt;=20"))</f>
         <v/>

</xml_diff>